<commit_message>
fix: unit test errors
</commit_message>
<xml_diff>
--- a/MetaboLights-Validations-v2.0.xlsx
+++ b/MetaboLights-Validations-v2.0.xlsx
@@ -15,7 +15,7 @@
     <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">Input!$A$1:$O$35</definedName>
     <definedName hidden="1" localSheetId="1" name="_xlnm._FilterDatabase">InvestigationFile!$A$1:$Q$85</definedName>
     <definedName hidden="1" localSheetId="2" name="_xlnm._FilterDatabase">SampleFile!$A$1:$Q$42</definedName>
-    <definedName hidden="1" localSheetId="3" name="_xlnm._FilterDatabase">AssayFile!$A$1:$Q$53</definedName>
+    <definedName hidden="1" localSheetId="3" name="_xlnm._FilterDatabase">AssayFile!$A$1:$Q$52</definedName>
     <definedName hidden="1" localSheetId="5" name="_xlnm._FilterDatabase">DataFiles!$A$1:$O$18</definedName>
     <definedName hidden="1" localSheetId="6" name="_xlnm._FilterDatabase">Summary!$A$1:$J$32</definedName>
   </definedNames>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3068" uniqueCount="972">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3058" uniqueCount="968">
   <si>
     <t>PHASE</t>
   </si>
@@ -2237,21 +2237,6 @@
     <t>All Derived Spectral Data File column values should have extension found in control list.</t>
   </si>
   <si>
-    <t>assays.chromatography</t>
-  </si>
-  <si>
-    <t>Column type</t>
-  </si>
-  <si>
-    <t>rule_a_200_600_001_01</t>
-  </si>
-  <si>
-    <t>Column Type column values are not same as assay file name.</t>
-  </si>
-  <si>
-    <t>if all values in Column Type are in a control list, technique name defined in control list should be in assay file name.</t>
-  </si>
-  <si>
     <t>assay.general</t>
   </si>
   <si>
@@ -2845,6 +2830,9 @@
   </si>
   <si>
     <t>There is no data transformation value errors in assay files.</t>
+  </si>
+  <si>
+    <t>assays.chromatography</t>
   </si>
   <si>
     <t>rule_a_200_600</t>
@@ -35021,112 +35009,63 @@
       <c r="AE51" s="67"/>
     </row>
     <row r="52">
-      <c r="A52" s="57" t="s">
+      <c r="A52" s="35" t="s">
         <v>394</v>
       </c>
-      <c r="B52" s="57"/>
-      <c r="C52" s="57"/>
-      <c r="D52" s="57" t="s">
-        <v>563</v>
-      </c>
-      <c r="E52" s="57" t="s">
-        <v>86</v>
-      </c>
-      <c r="F52" s="57" t="s">
+      <c r="B52" s="35"/>
+      <c r="C52" s="35"/>
+      <c r="D52" s="35" t="s">
+        <v>470</v>
+      </c>
+      <c r="E52" s="35" t="s">
+        <v>51</v>
+      </c>
+      <c r="F52" s="35" t="s">
         <v>720</v>
       </c>
-      <c r="G52" s="57" t="s">
+      <c r="G52" s="35" t="s">
+        <v>471</v>
+      </c>
+      <c r="H52" s="35" t="s">
         <v>721</v>
       </c>
-      <c r="H52" s="57" t="s">
-        <v>722</v>
-      </c>
-      <c r="I52" s="57" t="s">
+      <c r="I52" s="35" t="s">
         <v>36</v>
       </c>
-      <c r="J52" s="57" t="s">
-        <v>21</v>
-      </c>
-      <c r="K52" s="57" t="s">
-        <v>723</v>
-      </c>
-      <c r="L52" s="57" t="s">
-        <v>724</v>
-      </c>
-      <c r="M52" s="57"/>
-      <c r="N52" s="57"/>
-      <c r="O52" s="57"/>
-      <c r="P52" s="57"/>
-      <c r="Q52" s="57"/>
-      <c r="R52" s="67"/>
-      <c r="S52" s="67"/>
-      <c r="T52" s="67"/>
-      <c r="U52" s="67"/>
-      <c r="V52" s="67"/>
-      <c r="W52" s="67"/>
-      <c r="X52" s="67"/>
-      <c r="Y52" s="67"/>
-      <c r="Z52" s="67"/>
-      <c r="AA52" s="67"/>
-      <c r="AB52" s="67"/>
-      <c r="AC52" s="67"/>
-      <c r="AD52" s="67"/>
-      <c r="AE52" s="67"/>
+      <c r="J52" s="35" t="s">
+        <v>37</v>
+      </c>
+      <c r="K52" s="35" t="s">
+        <v>397</v>
+      </c>
+      <c r="L52" s="35" t="s">
+        <v>398</v>
+      </c>
+      <c r="M52" s="35"/>
+      <c r="N52" s="35"/>
+      <c r="O52" s="35" t="s">
+        <v>242</v>
+      </c>
+      <c r="P52" s="35"/>
+      <c r="Q52" s="35"/>
+      <c r="R52" s="37"/>
+      <c r="S52" s="37"/>
+      <c r="T52" s="37"/>
+      <c r="U52" s="37"/>
+      <c r="V52" s="37"/>
+      <c r="W52" s="37"/>
+      <c r="X52" s="37"/>
+      <c r="Y52" s="37"/>
+      <c r="Z52" s="37"/>
+      <c r="AA52" s="37"/>
+      <c r="AB52" s="37"/>
+      <c r="AC52" s="37"/>
+      <c r="AD52" s="37"/>
+      <c r="AE52" s="37"/>
     </row>
     <row r="53">
-      <c r="A53" s="35" t="s">
-        <v>394</v>
-      </c>
-      <c r="B53" s="35"/>
-      <c r="C53" s="35"/>
-      <c r="D53" s="35" t="s">
-        <v>470</v>
-      </c>
-      <c r="E53" s="35" t="s">
-        <v>51</v>
-      </c>
-      <c r="F53" s="35" t="s">
-        <v>725</v>
-      </c>
-      <c r="G53" s="35" t="s">
-        <v>471</v>
-      </c>
-      <c r="H53" s="35" t="s">
-        <v>726</v>
-      </c>
-      <c r="I53" s="35" t="s">
-        <v>36</v>
-      </c>
-      <c r="J53" s="35" t="s">
-        <v>37</v>
-      </c>
-      <c r="K53" s="35" t="s">
-        <v>397</v>
-      </c>
-      <c r="L53" s="35" t="s">
-        <v>398</v>
-      </c>
-      <c r="M53" s="35"/>
-      <c r="N53" s="35"/>
-      <c r="O53" s="35" t="s">
-        <v>242</v>
-      </c>
-      <c r="P53" s="35"/>
-      <c r="Q53" s="35"/>
-      <c r="R53" s="37"/>
-      <c r="S53" s="37"/>
-      <c r="T53" s="37"/>
-      <c r="U53" s="37"/>
-      <c r="V53" s="37"/>
-      <c r="W53" s="37"/>
-      <c r="X53" s="37"/>
-      <c r="Y53" s="37"/>
-      <c r="Z53" s="37"/>
-      <c r="AA53" s="37"/>
-      <c r="AB53" s="37"/>
-      <c r="AC53" s="37"/>
-      <c r="AD53" s="37"/>
-      <c r="AE53" s="37"/>
+      <c r="K53" s="51"/>
+      <c r="L53" s="51"/>
     </row>
     <row r="54">
       <c r="K54" s="51"/>
@@ -38820,12 +38759,8 @@
       <c r="K976" s="51"/>
       <c r="L976" s="51"/>
     </row>
-    <row r="977">
-      <c r="K977" s="51"/>
-      <c r="L977" s="51"/>
-    </row>
   </sheetData>
-  <autoFilter ref="$A$1:$Q$53"/>
+  <autoFilter ref="$A$1:$Q$52"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
@@ -38940,7 +38875,7 @@
         <v>18</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>727</v>
+        <v>722</v>
       </c>
       <c r="I2" s="5" t="s">
         <v>20</v>
@@ -38949,10 +38884,10 @@
         <v>21</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>728</v>
+        <v>723</v>
       </c>
       <c r="L2" s="5" t="s">
-        <v>729</v>
+        <v>724</v>
       </c>
       <c r="M2" s="5"/>
       <c r="N2" s="5"/>
@@ -38979,7 +38914,7 @@
         <v>18</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>730</v>
+        <v>725</v>
       </c>
       <c r="I3" s="5" t="s">
         <v>20</v>
@@ -38988,15 +38923,15 @@
         <v>21</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>731</v>
+        <v>726</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>731</v>
+        <v>726</v>
       </c>
       <c r="M3" s="5"/>
       <c r="N3" s="5"/>
       <c r="O3" s="8" t="s">
-        <v>732</v>
+        <v>727</v>
       </c>
       <c r="P3" s="8"/>
       <c r="Q3" s="8"/>
@@ -39020,7 +38955,7 @@
         <v>18</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>733</v>
+        <v>728</v>
       </c>
       <c r="I4" s="5" t="s">
         <v>20</v>
@@ -39029,10 +38964,10 @@
         <v>21</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>734</v>
+        <v>729</v>
       </c>
       <c r="L4" s="5" t="s">
-        <v>735</v>
+        <v>730</v>
       </c>
       <c r="M4" s="5"/>
       <c r="N4" s="5"/>
@@ -39073,7 +39008,7 @@
         <v>18</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>736</v>
+        <v>731</v>
       </c>
       <c r="I5" s="5" t="s">
         <v>20</v>
@@ -39082,10 +39017,10 @@
         <v>21</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>737</v>
+        <v>732</v>
       </c>
       <c r="L5" s="5" t="s">
-        <v>738</v>
+        <v>733</v>
       </c>
       <c r="M5" s="5"/>
       <c r="N5" s="5"/>
@@ -39126,7 +39061,7 @@
         <v>18</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>739</v>
+        <v>734</v>
       </c>
       <c r="I6" s="5" t="s">
         <v>36</v>
@@ -39135,17 +39070,17 @@
         <v>21</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>740</v>
+        <v>735</v>
       </c>
       <c r="L6" s="5" t="s">
-        <v>741</v>
+        <v>736</v>
       </c>
       <c r="M6" s="5"/>
       <c r="N6" s="5" t="s">
-        <v>742</v>
+        <v>737</v>
       </c>
       <c r="O6" s="48" t="s">
-        <v>743</v>
+        <v>738</v>
       </c>
       <c r="P6" s="48"/>
       <c r="Q6" s="48"/>
@@ -39183,7 +39118,7 @@
         <v>18</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>744</v>
+        <v>739</v>
       </c>
       <c r="I7" s="5" t="s">
         <v>36</v>
@@ -39192,14 +39127,14 @@
         <v>21</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>745</v>
+        <v>740</v>
       </c>
       <c r="L7" s="5" t="s">
-        <v>746</v>
+        <v>741</v>
       </c>
       <c r="M7" s="5"/>
       <c r="N7" s="5" t="s">
-        <v>747</v>
+        <v>742</v>
       </c>
       <c r="O7" s="48"/>
       <c r="P7" s="48"/>
@@ -39238,7 +39173,7 @@
         <v>18</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>748</v>
+        <v>743</v>
       </c>
       <c r="I8" s="5" t="s">
         <v>20</v>
@@ -39247,15 +39182,15 @@
         <v>21</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>749</v>
+        <v>744</v>
       </c>
       <c r="L8" s="5" t="s">
-        <v>750</v>
+        <v>745</v>
       </c>
       <c r="M8" s="5"/>
       <c r="N8" s="5"/>
       <c r="O8" s="48" t="s">
-        <v>751</v>
+        <v>746</v>
       </c>
       <c r="P8" s="48"/>
       <c r="Q8" s="48"/>
@@ -39293,7 +39228,7 @@
         <v>18</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>752</v>
+        <v>747</v>
       </c>
       <c r="I9" s="5" t="s">
         <v>20</v>
@@ -39346,7 +39281,7 @@
         <v>18</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>753</v>
+        <v>748</v>
       </c>
       <c r="I10" s="5" t="s">
         <v>20</v>
@@ -39355,10 +39290,10 @@
         <v>21</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>754</v>
+        <v>749</v>
       </c>
       <c r="L10" s="5" t="s">
-        <v>755</v>
+        <v>750</v>
       </c>
       <c r="M10" s="5"/>
       <c r="N10" s="5"/>
@@ -39399,7 +39334,7 @@
         <v>18</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>756</v>
+        <v>751</v>
       </c>
       <c r="I11" s="5" t="s">
         <v>20</v>
@@ -39408,10 +39343,10 @@
         <v>37</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>757</v>
+        <v>752</v>
       </c>
       <c r="L11" s="5" t="s">
-        <v>758</v>
+        <v>753</v>
       </c>
       <c r="M11" s="5"/>
       <c r="N11" s="5"/>
@@ -39435,7 +39370,7 @@
     </row>
     <row r="12">
       <c r="A12" s="5" t="s">
-        <v>759</v>
+        <v>754</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -39452,7 +39387,7 @@
         <v>471</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>760</v>
+        <v>755</v>
       </c>
       <c r="I12" s="5" t="s">
         <v>20</v>
@@ -39461,10 +39396,10 @@
         <v>37</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>761</v>
+        <v>756</v>
       </c>
       <c r="L12" s="5" t="s">
-        <v>762</v>
+        <v>757</v>
       </c>
       <c r="M12" s="5"/>
       <c r="N12" s="5"/>
@@ -39488,7 +39423,7 @@
     </row>
     <row r="13">
       <c r="A13" s="5" t="s">
-        <v>759</v>
+        <v>754</v>
       </c>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
@@ -39505,7 +39440,7 @@
         <v>471</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>763</v>
+        <v>758</v>
       </c>
       <c r="I13" s="5" t="s">
         <v>20</v>
@@ -39514,15 +39449,15 @@
         <v>37</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>764</v>
+        <v>759</v>
       </c>
       <c r="L13" s="5" t="s">
-        <v>765</v>
+        <v>760</v>
       </c>
       <c r="M13" s="5"/>
       <c r="N13" s="5"/>
       <c r="O13" s="48" t="s">
-        <v>766</v>
+        <v>761</v>
       </c>
       <c r="P13" s="48"/>
       <c r="Q13" s="48"/>
@@ -39543,7 +39478,7 @@
     </row>
     <row r="14">
       <c r="A14" s="5" t="s">
-        <v>759</v>
+        <v>754</v>
       </c>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
@@ -39560,7 +39495,7 @@
         <v>471</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>767</v>
+        <v>762</v>
       </c>
       <c r="I14" s="5" t="s">
         <v>20</v>
@@ -39572,7 +39507,7 @@
         <v>529</v>
       </c>
       <c r="L14" s="5" t="s">
-        <v>768</v>
+        <v>763</v>
       </c>
       <c r="M14" s="5"/>
       <c r="N14" s="5"/>
@@ -39596,7 +39531,7 @@
     </row>
     <row r="15">
       <c r="A15" s="5" t="s">
-        <v>759</v>
+        <v>754</v>
       </c>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
@@ -39613,7 +39548,7 @@
         <v>471</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>769</v>
+        <v>764</v>
       </c>
       <c r="I15" s="5" t="s">
         <v>20</v>
@@ -39625,7 +39560,7 @@
         <v>534</v>
       </c>
       <c r="L15" s="5" t="s">
-        <v>770</v>
+        <v>765</v>
       </c>
       <c r="M15" s="5"/>
       <c r="N15" s="5"/>
@@ -39649,7 +39584,7 @@
     </row>
     <row r="16">
       <c r="A16" s="5" t="s">
-        <v>759</v>
+        <v>754</v>
       </c>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
@@ -39660,13 +39595,13 @@
         <v>116</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>771</v>
+        <v>766</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>772</v>
+        <v>767</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>773</v>
+        <v>768</v>
       </c>
       <c r="I16" s="5" t="s">
         <v>20</v>
@@ -39675,17 +39610,17 @@
         <v>37</v>
       </c>
       <c r="K16" s="5" t="s">
-        <v>774</v>
+        <v>769</v>
       </c>
       <c r="L16" s="5" t="s">
-        <v>775</v>
+        <v>770</v>
       </c>
       <c r="M16" s="5"/>
       <c r="N16" s="5" t="s">
-        <v>776</v>
+        <v>771</v>
       </c>
       <c r="O16" s="48" t="s">
-        <v>777</v>
+        <v>772</v>
       </c>
       <c r="P16" s="48"/>
       <c r="Q16" s="48"/>
@@ -39706,7 +39641,7 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>759</v>
+        <v>754</v>
       </c>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
@@ -39717,13 +39652,13 @@
         <v>116</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>771</v>
+        <v>766</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>778</v>
+        <v>773</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>779</v>
+        <v>774</v>
       </c>
       <c r="I17" s="5" t="s">
         <v>20</v>
@@ -39732,14 +39667,14 @@
         <v>37</v>
       </c>
       <c r="K17" s="5" t="s">
-        <v>780</v>
+        <v>775</v>
       </c>
       <c r="L17" s="5" t="s">
-        <v>781</v>
+        <v>776</v>
       </c>
       <c r="M17" s="5"/>
       <c r="N17" s="5" t="s">
-        <v>776</v>
+        <v>771</v>
       </c>
       <c r="O17" s="48"/>
       <c r="P17" s="48"/>
@@ -39761,7 +39696,7 @@
     </row>
     <row r="18">
       <c r="A18" s="5" t="s">
-        <v>759</v>
+        <v>754</v>
       </c>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
@@ -39772,13 +39707,13 @@
         <v>116</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>771</v>
+        <v>766</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>778</v>
+        <v>773</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>782</v>
+        <v>777</v>
       </c>
       <c r="I18" s="5" t="s">
         <v>36</v>
@@ -39787,14 +39722,14 @@
         <v>37</v>
       </c>
       <c r="K18" s="5" t="s">
-        <v>783</v>
+        <v>778</v>
       </c>
       <c r="L18" s="5" t="s">
-        <v>784</v>
+        <v>779</v>
       </c>
       <c r="M18" s="5"/>
       <c r="N18" s="5" t="s">
-        <v>776</v>
+        <v>771</v>
       </c>
       <c r="O18" s="48"/>
       <c r="P18" s="48"/>
@@ -39816,7 +39751,7 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>759</v>
+        <v>754</v>
       </c>
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
@@ -39827,13 +39762,13 @@
         <v>116</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>785</v>
+        <v>780</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>786</v>
+        <v>781</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>787</v>
+        <v>782</v>
       </c>
       <c r="I19" s="5" t="s">
         <v>36</v>
@@ -39842,17 +39777,17 @@
         <v>21</v>
       </c>
       <c r="K19" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="L19" s="5" t="s">
-        <v>789</v>
+        <v>784</v>
       </c>
       <c r="M19" s="5"/>
       <c r="N19" s="5" t="s">
-        <v>790</v>
+        <v>785</v>
       </c>
       <c r="O19" s="48" t="s">
-        <v>777</v>
+        <v>772</v>
       </c>
       <c r="P19" s="48"/>
       <c r="Q19" s="48"/>
@@ -39873,7 +39808,7 @@
     </row>
     <row r="20">
       <c r="A20" s="5" t="s">
-        <v>759</v>
+        <v>754</v>
       </c>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
@@ -39884,13 +39819,13 @@
         <v>116</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>785</v>
+        <v>780</v>
       </c>
       <c r="G20" s="5" t="s">
+        <v>781</v>
+      </c>
+      <c r="H20" s="5" t="s">
         <v>786</v>
-      </c>
-      <c r="H20" s="5" t="s">
-        <v>791</v>
       </c>
       <c r="I20" s="5" t="s">
         <v>36</v>
@@ -39899,14 +39834,14 @@
         <v>37</v>
       </c>
       <c r="K20" s="5" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="L20" s="5" t="s">
-        <v>793</v>
+        <v>788</v>
       </c>
       <c r="M20" s="5"/>
       <c r="N20" s="5" t="s">
-        <v>790</v>
+        <v>785</v>
       </c>
       <c r="O20" s="48"/>
       <c r="P20" s="48"/>
@@ -39928,7 +39863,7 @@
     </row>
     <row r="21">
       <c r="A21" s="5" t="s">
-        <v>759</v>
+        <v>754</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -39939,13 +39874,13 @@
         <v>116</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>785</v>
+        <v>780</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>794</v>
+        <v>789</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>795</v>
+        <v>790</v>
       </c>
       <c r="I21" s="5" t="s">
         <v>36</v>
@@ -39954,14 +39889,14 @@
         <v>21</v>
       </c>
       <c r="K21" s="5" t="s">
-        <v>796</v>
+        <v>791</v>
       </c>
       <c r="L21" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="M21" s="5"/>
       <c r="N21" s="5" t="s">
-        <v>790</v>
+        <v>785</v>
       </c>
       <c r="O21" s="48"/>
       <c r="P21" s="48"/>
@@ -43937,22 +43872,22 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>798</v>
+        <v>793</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>16</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>799</v>
+        <v>794</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>800</v>
+        <v>795</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>801</v>
+        <v>796</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>802</v>
+        <v>797</v>
       </c>
       <c r="G2" s="5" t="s">
         <v>20</v>
@@ -43961,13 +43896,13 @@
         <v>21</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>803</v>
+        <v>798</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>804</v>
+        <v>799</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>805</v>
+        <v>800</v>
       </c>
       <c r="L2" s="5"/>
       <c r="M2" s="69"/>
@@ -43991,20 +43926,20 @@
     </row>
     <row r="3">
       <c r="A3" s="5" t="s">
-        <v>798</v>
+        <v>793</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5" t="s">
-        <v>799</v>
+        <v>794</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>800</v>
+        <v>795</v>
       </c>
       <c r="E3" s="5" t="s">
+        <v>796</v>
+      </c>
+      <c r="F3" s="5" t="s">
         <v>801</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>806</v>
       </c>
       <c r="G3" s="5" t="s">
         <v>20</v>
@@ -44013,13 +43948,13 @@
         <v>21</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>807</v>
+        <v>802</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>808</v>
+        <v>803</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>809</v>
+        <v>804</v>
       </c>
       <c r="L3" s="5"/>
       <c r="M3" s="69"/>
@@ -44028,20 +43963,20 @@
     </row>
     <row r="4">
       <c r="A4" s="5" t="s">
-        <v>798</v>
+        <v>793</v>
       </c>
       <c r="B4" s="5"/>
       <c r="C4" s="5" t="s">
-        <v>799</v>
+        <v>794</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>800</v>
+        <v>795</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>810</v>
+        <v>805</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>811</v>
+        <v>806</v>
       </c>
       <c r="G4" s="5" t="s">
         <v>20</v>
@@ -44050,13 +43985,13 @@
         <v>37</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>812</v>
+        <v>807</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>813</v>
+        <v>808</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>814</v>
+        <v>809</v>
       </c>
       <c r="L4" s="5"/>
       <c r="M4" s="69"/>
@@ -44065,20 +44000,20 @@
     </row>
     <row r="5">
       <c r="A5" s="5" t="s">
-        <v>798</v>
+        <v>793</v>
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="5" t="s">
-        <v>815</v>
+        <v>810</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>800</v>
+        <v>795</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>810</v>
+        <v>805</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>816</v>
+        <v>811</v>
       </c>
       <c r="G5" s="5" t="s">
         <v>20</v>
@@ -44087,13 +44022,13 @@
         <v>21</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>817</v>
+        <v>812</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>818</v>
+        <v>813</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>819</v>
+        <v>814</v>
       </c>
       <c r="L5" s="5"/>
       <c r="M5" s="69"/>
@@ -44102,20 +44037,20 @@
     </row>
     <row r="6">
       <c r="A6" s="20" t="s">
-        <v>798</v>
+        <v>793</v>
       </c>
       <c r="B6" s="20"/>
       <c r="C6" s="20" t="s">
-        <v>799</v>
+        <v>794</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>800</v>
+        <v>795</v>
       </c>
       <c r="E6" s="20" t="s">
-        <v>810</v>
+        <v>805</v>
       </c>
       <c r="F6" s="20" t="s">
-        <v>820</v>
+        <v>815</v>
       </c>
       <c r="G6" s="20" t="s">
         <v>20</v>
@@ -44124,13 +44059,13 @@
         <v>37</v>
       </c>
       <c r="I6" s="20" t="s">
-        <v>821</v>
+        <v>816</v>
       </c>
       <c r="J6" s="20" t="s">
-        <v>822</v>
+        <v>817</v>
       </c>
       <c r="K6" s="20" t="s">
-        <v>823</v>
+        <v>818</v>
       </c>
       <c r="L6" s="20"/>
       <c r="M6" s="70"/>
@@ -44154,20 +44089,20 @@
     </row>
     <row r="7">
       <c r="A7" s="71" t="s">
-        <v>798</v>
+        <v>793</v>
       </c>
       <c r="B7" s="71"/>
       <c r="C7" s="71" t="s">
-        <v>799</v>
+        <v>794</v>
       </c>
       <c r="D7" s="71" t="s">
-        <v>800</v>
+        <v>795</v>
       </c>
       <c r="E7" s="71" t="s">
-        <v>810</v>
+        <v>805</v>
       </c>
       <c r="F7" s="71" t="s">
-        <v>824</v>
+        <v>819</v>
       </c>
       <c r="G7" s="71" t="s">
         <v>20</v>
@@ -44176,16 +44111,16 @@
         <v>37</v>
       </c>
       <c r="I7" s="71" t="s">
-        <v>825</v>
+        <v>820</v>
       </c>
       <c r="J7" s="71" t="s">
-        <v>826</v>
+        <v>821</v>
       </c>
       <c r="K7" s="71" t="s">
-        <v>827</v>
+        <v>822</v>
       </c>
       <c r="L7" s="71" t="s">
-        <v>828</v>
+        <v>823</v>
       </c>
       <c r="M7" s="72"/>
       <c r="N7" s="72"/>
@@ -44208,20 +44143,20 @@
     </row>
     <row r="8">
       <c r="A8" s="5" t="s">
-        <v>798</v>
+        <v>793</v>
       </c>
       <c r="B8" s="5"/>
       <c r="C8" s="5" t="s">
-        <v>799</v>
+        <v>794</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>800</v>
+        <v>795</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>829</v>
+        <v>824</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>830</v>
+        <v>825</v>
       </c>
       <c r="G8" s="5" t="s">
         <v>20</v>
@@ -44230,13 +44165,13 @@
         <v>37</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>831</v>
+        <v>826</v>
       </c>
       <c r="J8" s="5" t="s">
-        <v>832</v>
+        <v>827</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>814</v>
+        <v>809</v>
       </c>
       <c r="L8" s="5"/>
       <c r="M8" s="69"/>
@@ -44245,35 +44180,35 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="s">
-        <v>798</v>
+        <v>793</v>
       </c>
       <c r="B9" s="5"/>
       <c r="C9" s="5" t="s">
-        <v>799</v>
+        <v>794</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>800</v>
+        <v>795</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>681</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>833</v>
+        <v>828</v>
       </c>
       <c r="G9" s="5" t="s">
         <v>36</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>834</v>
+        <v>829</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>835</v>
+        <v>830</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>836</v>
+        <v>831</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>837</v>
+        <v>832</v>
       </c>
       <c r="L9" s="5"/>
       <c r="M9" s="69"/>
@@ -44282,35 +44217,35 @@
     </row>
     <row r="10" ht="73.5" customHeight="1">
       <c r="A10" s="5" t="s">
-        <v>798</v>
+        <v>793</v>
       </c>
       <c r="B10" s="5"/>
       <c r="C10" s="5" t="s">
-        <v>799</v>
+        <v>794</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>800</v>
+        <v>795</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>716</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>838</v>
+        <v>833</v>
       </c>
       <c r="G10" s="5" t="s">
         <v>36</v>
       </c>
       <c r="H10" s="5" t="s">
+        <v>829</v>
+      </c>
+      <c r="I10" s="5" t="s">
         <v>834</v>
       </c>
-      <c r="I10" s="5" t="s">
-        <v>839</v>
-      </c>
       <c r="J10" s="5" t="s">
-        <v>840</v>
+        <v>835</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>841</v>
+        <v>836</v>
       </c>
       <c r="L10" s="5"/>
       <c r="M10" s="69"/>
@@ -44319,35 +44254,35 @@
     </row>
     <row r="11">
       <c r="A11" s="5" t="s">
-        <v>798</v>
+        <v>793</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="5" t="s">
-        <v>815</v>
+        <v>810</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>800</v>
+        <v>795</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>18</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>842</v>
+        <v>837</v>
       </c>
       <c r="G11" s="5" t="s">
         <v>20</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>843</v>
+        <v>838</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>844</v>
+        <v>839</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>845</v>
+        <v>840</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>846</v>
+        <v>841</v>
       </c>
       <c r="L11" s="5"/>
       <c r="M11" s="69"/>
@@ -44356,20 +44291,20 @@
     </row>
     <row r="12">
       <c r="A12" s="5" t="s">
-        <v>798</v>
+        <v>793</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5" t="s">
-        <v>815</v>
+        <v>810</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>800</v>
+        <v>795</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>18</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>847</v>
+        <v>842</v>
       </c>
       <c r="G12" s="5" t="s">
         <v>36</v>
@@ -44378,13 +44313,13 @@
         <v>37</v>
       </c>
       <c r="I12" s="5" t="s">
-        <v>848</v>
+        <v>843</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>849</v>
+        <v>844</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>850</v>
+        <v>845</v>
       </c>
       <c r="L12" s="5"/>
       <c r="M12" s="69"/>
@@ -44393,20 +44328,20 @@
     </row>
     <row r="13">
       <c r="A13" s="5" t="s">
-        <v>798</v>
+        <v>793</v>
       </c>
       <c r="B13" s="5"/>
       <c r="C13" s="5" t="s">
-        <v>815</v>
+        <v>810</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>800</v>
+        <v>795</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>18</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>851</v>
+        <v>846</v>
       </c>
       <c r="G13" s="5" t="s">
         <v>36</v>
@@ -44415,13 +44350,13 @@
         <v>21</v>
       </c>
       <c r="I13" s="5" t="s">
-        <v>852</v>
+        <v>847</v>
       </c>
       <c r="J13" s="5" t="s">
-        <v>853</v>
+        <v>848</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>854</v>
+        <v>849</v>
       </c>
       <c r="L13" s="5"/>
       <c r="M13" s="69"/>
@@ -44430,20 +44365,20 @@
     </row>
     <row r="14">
       <c r="A14" s="5" t="s">
-        <v>798</v>
+        <v>793</v>
       </c>
       <c r="B14" s="5"/>
       <c r="C14" s="5" t="s">
-        <v>815</v>
+        <v>810</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>800</v>
+        <v>795</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>18</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>855</v>
+        <v>850</v>
       </c>
       <c r="G14" s="5" t="s">
         <v>36</v>
@@ -44452,13 +44387,13 @@
         <v>21</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>856</v>
+        <v>851</v>
       </c>
       <c r="J14" s="5" t="s">
-        <v>857</v>
+        <v>852</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>858</v>
+        <v>853</v>
       </c>
       <c r="L14" s="5"/>
       <c r="M14" s="69"/>
@@ -44467,20 +44402,20 @@
     </row>
     <row r="15">
       <c r="A15" s="5" t="s">
-        <v>798</v>
+        <v>793</v>
       </c>
       <c r="B15" s="5"/>
       <c r="C15" s="5" t="s">
-        <v>815</v>
+        <v>810</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>800</v>
+        <v>795</v>
       </c>
       <c r="E15" s="5" t="s">
         <v>18</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>859</v>
+        <v>854</v>
       </c>
       <c r="G15" s="5" t="s">
         <v>20</v>
@@ -44489,13 +44424,13 @@
         <v>21</v>
       </c>
       <c r="I15" s="5" t="s">
-        <v>860</v>
+        <v>855</v>
       </c>
       <c r="J15" s="5" t="s">
-        <v>861</v>
+        <v>856</v>
       </c>
       <c r="K15" s="5" t="s">
-        <v>862</v>
+        <v>857</v>
       </c>
       <c r="L15" s="5"/>
       <c r="M15" s="69"/>
@@ -44504,20 +44439,20 @@
     </row>
     <row r="16">
       <c r="A16" s="5" t="s">
-        <v>798</v>
+        <v>793</v>
       </c>
       <c r="B16" s="5"/>
       <c r="C16" s="5" t="s">
-        <v>815</v>
+        <v>810</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>800</v>
+        <v>795</v>
       </c>
       <c r="E16" s="5" t="s">
         <v>18</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>863</v>
+        <v>858</v>
       </c>
       <c r="G16" s="5" t="s">
         <v>20</v>
@@ -44526,10 +44461,10 @@
         <v>37</v>
       </c>
       <c r="I16" s="5" t="s">
-        <v>864</v>
+        <v>859</v>
       </c>
       <c r="J16" s="5" t="s">
-        <v>865</v>
+        <v>860</v>
       </c>
       <c r="K16" s="5"/>
       <c r="L16" s="5"/>
@@ -44539,20 +44474,20 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>798</v>
+        <v>793</v>
       </c>
       <c r="B17" s="5"/>
       <c r="C17" s="5" t="s">
-        <v>815</v>
+        <v>810</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>800</v>
+        <v>795</v>
       </c>
       <c r="E17" s="5" t="s">
         <v>18</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>866</v>
+        <v>861</v>
       </c>
       <c r="G17" s="5" t="s">
         <v>20</v>
@@ -44561,10 +44496,10 @@
         <v>21</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>867</v>
+        <v>862</v>
       </c>
       <c r="J17" s="5" t="s">
-        <v>868</v>
+        <v>863</v>
       </c>
       <c r="K17" s="5"/>
       <c r="L17" s="5"/>
@@ -44574,20 +44509,20 @@
     </row>
     <row r="18">
       <c r="A18" s="5" t="s">
-        <v>798</v>
+        <v>793</v>
       </c>
       <c r="B18" s="5"/>
       <c r="C18" s="5" t="s">
-        <v>815</v>
+        <v>810</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>800</v>
+        <v>795</v>
       </c>
       <c r="E18" s="5" t="s">
         <v>18</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>869</v>
+        <v>864</v>
       </c>
       <c r="G18" s="5" t="s">
         <v>20</v>
@@ -44596,16 +44531,16 @@
         <v>37</v>
       </c>
       <c r="I18" s="5" t="s">
-        <v>870</v>
+        <v>865</v>
       </c>
       <c r="J18" s="5" t="s">
-        <v>871</v>
+        <v>866</v>
       </c>
       <c r="K18" s="5" t="s">
-        <v>872</v>
+        <v>867</v>
       </c>
       <c r="L18" s="5" t="s">
-        <v>873</v>
+        <v>868</v>
       </c>
       <c r="M18" s="69"/>
       <c r="N18" s="69"/>
@@ -48557,15 +48492,15 @@
       </c>
       <c r="E2" s="7"/>
       <c r="F2" s="7" t="s">
-        <v>874</v>
+        <v>869</v>
       </c>
       <c r="G2" s="6"/>
       <c r="H2" s="7"/>
       <c r="I2" s="7" t="s">
-        <v>875</v>
+        <v>870</v>
       </c>
       <c r="J2" s="7" t="s">
-        <v>876</v>
+        <v>871</v>
       </c>
     </row>
     <row r="3">
@@ -48577,19 +48512,19 @@
         <v>17</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>877</v>
+        <v>872</v>
       </c>
       <c r="E3" s="7"/>
       <c r="F3" s="7" t="s">
-        <v>878</v>
+        <v>873</v>
       </c>
       <c r="G3" s="7"/>
       <c r="H3" s="7"/>
       <c r="I3" s="7" t="s">
-        <v>879</v>
+        <v>874</v>
       </c>
       <c r="J3" s="7" t="s">
-        <v>880</v>
+        <v>875</v>
       </c>
     </row>
     <row r="4">
@@ -48601,19 +48536,19 @@
         <v>51</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>881</v>
+        <v>876</v>
       </c>
       <c r="E4" s="7"/>
       <c r="F4" s="7" t="s">
-        <v>882</v>
+        <v>877</v>
       </c>
       <c r="G4" s="7"/>
       <c r="H4" s="7"/>
       <c r="I4" s="7" t="s">
-        <v>883</v>
+        <v>878</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>884</v>
+        <v>879</v>
       </c>
     </row>
     <row r="5">
@@ -48625,19 +48560,19 @@
         <v>86</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>885</v>
+        <v>880</v>
       </c>
       <c r="E5" s="7"/>
       <c r="F5" s="7" t="s">
-        <v>886</v>
+        <v>881</v>
       </c>
       <c r="G5" s="7"/>
       <c r="H5" s="7"/>
       <c r="I5" s="7" t="s">
-        <v>887</v>
+        <v>882</v>
       </c>
       <c r="J5" s="7" t="s">
-        <v>888</v>
+        <v>883</v>
       </c>
     </row>
     <row r="6">
@@ -48653,15 +48588,15 @@
       </c>
       <c r="E6" s="7"/>
       <c r="F6" s="7" t="s">
-        <v>889</v>
+        <v>884</v>
       </c>
       <c r="G6" s="7"/>
       <c r="H6" s="7"/>
       <c r="I6" s="7" t="s">
-        <v>890</v>
+        <v>885</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>891</v>
+        <v>886</v>
       </c>
     </row>
     <row r="7">
@@ -48677,15 +48612,15 @@
       </c>
       <c r="E7" s="7"/>
       <c r="F7" s="7" t="s">
-        <v>892</v>
+        <v>887</v>
       </c>
       <c r="G7" s="7"/>
       <c r="H7" s="7"/>
       <c r="I7" s="7" t="s">
-        <v>893</v>
+        <v>888</v>
       </c>
       <c r="J7" s="7" t="s">
-        <v>894</v>
+        <v>889</v>
       </c>
     </row>
     <row r="8">
@@ -48697,19 +48632,19 @@
         <v>86</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>895</v>
+        <v>890</v>
       </c>
       <c r="E8" s="7"/>
       <c r="F8" s="7" t="s">
-        <v>896</v>
+        <v>891</v>
       </c>
       <c r="G8" s="7"/>
       <c r="H8" s="7"/>
       <c r="I8" s="7" t="s">
-        <v>897</v>
+        <v>892</v>
       </c>
       <c r="J8" s="7" t="s">
-        <v>898</v>
+        <v>893</v>
       </c>
     </row>
     <row r="9">
@@ -48721,19 +48656,19 @@
         <v>86</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>899</v>
+        <v>894</v>
       </c>
       <c r="E9" s="7"/>
       <c r="F9" s="7" t="s">
-        <v>900</v>
+        <v>895</v>
       </c>
       <c r="G9" s="7"/>
       <c r="H9" s="7"/>
       <c r="I9" s="7" t="s">
-        <v>901</v>
+        <v>896</v>
       </c>
       <c r="J9" s="7" t="s">
-        <v>902</v>
+        <v>897</v>
       </c>
     </row>
     <row r="10">
@@ -48749,15 +48684,15 @@
       </c>
       <c r="E10" s="7"/>
       <c r="F10" s="7" t="s">
-        <v>903</v>
+        <v>898</v>
       </c>
       <c r="G10" s="7"/>
       <c r="H10" s="7"/>
       <c r="I10" s="7" t="s">
-        <v>904</v>
+        <v>899</v>
       </c>
       <c r="J10" s="7" t="s">
-        <v>905</v>
+        <v>900</v>
       </c>
     </row>
     <row r="11">
@@ -48773,15 +48708,15 @@
       </c>
       <c r="E11" s="7"/>
       <c r="F11" s="7" t="s">
-        <v>906</v>
+        <v>901</v>
       </c>
       <c r="G11" s="7"/>
       <c r="H11" s="7"/>
       <c r="I11" s="7" t="s">
-        <v>907</v>
+        <v>902</v>
       </c>
       <c r="J11" s="7" t="s">
-        <v>908</v>
+        <v>903</v>
       </c>
     </row>
     <row r="12">
@@ -48797,15 +48732,15 @@
       </c>
       <c r="E12" s="7"/>
       <c r="F12" s="7" t="s">
-        <v>909</v>
+        <v>904</v>
       </c>
       <c r="G12" s="7"/>
       <c r="H12" s="7"/>
       <c r="I12" s="7" t="s">
-        <v>910</v>
+        <v>905</v>
       </c>
       <c r="J12" s="7" t="s">
-        <v>911</v>
+        <v>906</v>
       </c>
     </row>
     <row r="13">
@@ -48821,15 +48756,15 @@
       </c>
       <c r="E13" s="7"/>
       <c r="F13" s="7" t="s">
-        <v>912</v>
+        <v>907</v>
       </c>
       <c r="G13" s="7"/>
       <c r="H13" s="7"/>
       <c r="I13" s="6" t="s">
-        <v>913</v>
+        <v>908</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>914</v>
+        <v>909</v>
       </c>
     </row>
     <row r="14">
@@ -48841,67 +48776,67 @@
         <v>86</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>720</v>
+        <v>910</v>
       </c>
       <c r="E14" s="7"/>
       <c r="F14" s="6" t="s">
-        <v>915</v>
+        <v>911</v>
       </c>
       <c r="G14" s="7"/>
       <c r="H14" s="7"/>
       <c r="I14" s="6" t="s">
-        <v>916</v>
+        <v>912</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>917</v>
+        <v>913</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="s">
-        <v>798</v>
+        <v>793</v>
       </c>
       <c r="B15" s="7"/>
       <c r="C15" s="7" t="s">
-        <v>918</v>
+        <v>914</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>800</v>
+        <v>795</v>
       </c>
       <c r="E15" s="7"/>
       <c r="F15" s="7" t="s">
-        <v>919</v>
+        <v>915</v>
       </c>
       <c r="G15" s="7"/>
       <c r="H15" s="7"/>
       <c r="I15" s="7" t="s">
-        <v>920</v>
+        <v>916</v>
       </c>
       <c r="J15" s="7" t="s">
-        <v>921</v>
+        <v>917</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="s">
-        <v>798</v>
+        <v>793</v>
       </c>
       <c r="B16" s="7"/>
       <c r="C16" s="7" t="s">
+        <v>914</v>
+      </c>
+      <c r="D16" s="6" t="s">
         <v>918</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>922</v>
       </c>
       <c r="E16" s="7"/>
       <c r="F16" s="7" t="s">
-        <v>923</v>
+        <v>919</v>
       </c>
       <c r="G16" s="7"/>
       <c r="H16" s="7"/>
       <c r="I16" s="7" t="s">
-        <v>924</v>
+        <v>920</v>
       </c>
       <c r="J16" s="7" t="s">
-        <v>925</v>
+        <v>921</v>
       </c>
     </row>
     <row r="17">
@@ -48917,15 +48852,15 @@
       </c>
       <c r="E17" s="7"/>
       <c r="F17" s="7" t="s">
-        <v>926</v>
+        <v>922</v>
       </c>
       <c r="G17" s="7"/>
       <c r="H17" s="7"/>
       <c r="I17" s="7" t="s">
-        <v>927</v>
+        <v>923</v>
       </c>
       <c r="J17" s="7" t="s">
-        <v>928</v>
+        <v>924</v>
       </c>
     </row>
     <row r="18">
@@ -48941,15 +48876,15 @@
       </c>
       <c r="E18" s="7"/>
       <c r="F18" s="7" t="s">
-        <v>929</v>
+        <v>925</v>
       </c>
       <c r="G18" s="7"/>
       <c r="H18" s="7"/>
       <c r="I18" s="7" t="s">
-        <v>930</v>
+        <v>926</v>
       </c>
       <c r="J18" s="7" t="s">
-        <v>931</v>
+        <v>927</v>
       </c>
     </row>
     <row r="19">
@@ -48965,15 +48900,15 @@
       </c>
       <c r="E19" s="7"/>
       <c r="F19" s="7" t="s">
-        <v>932</v>
+        <v>928</v>
       </c>
       <c r="G19" s="7"/>
       <c r="H19" s="7"/>
       <c r="I19" s="7" t="s">
-        <v>933</v>
+        <v>929</v>
       </c>
       <c r="J19" s="7" t="s">
-        <v>934</v>
+        <v>930</v>
       </c>
     </row>
     <row r="20">
@@ -48989,15 +48924,15 @@
       </c>
       <c r="E20" s="7"/>
       <c r="F20" s="7" t="s">
-        <v>935</v>
+        <v>931</v>
       </c>
       <c r="G20" s="7"/>
       <c r="H20" s="7"/>
       <c r="I20" s="7" t="s">
-        <v>936</v>
+        <v>932</v>
       </c>
       <c r="J20" s="7" t="s">
-        <v>898</v>
+        <v>893</v>
       </c>
     </row>
     <row r="21">
@@ -49013,15 +48948,15 @@
       </c>
       <c r="E21" s="7"/>
       <c r="F21" s="7" t="s">
-        <v>937</v>
+        <v>933</v>
       </c>
       <c r="G21" s="7"/>
       <c r="H21" s="7"/>
       <c r="I21" s="7" t="s">
-        <v>938</v>
+        <v>934</v>
       </c>
       <c r="J21" s="7" t="s">
-        <v>939</v>
+        <v>935</v>
       </c>
     </row>
     <row r="22">
@@ -49037,15 +48972,15 @@
       </c>
       <c r="E22" s="7"/>
       <c r="F22" s="7" t="s">
-        <v>940</v>
+        <v>936</v>
       </c>
       <c r="G22" s="7"/>
       <c r="H22" s="7"/>
       <c r="I22" s="7" t="s">
-        <v>941</v>
+        <v>937</v>
       </c>
       <c r="J22" s="7" t="s">
-        <v>942</v>
+        <v>938</v>
       </c>
     </row>
     <row r="23">
@@ -49061,15 +48996,15 @@
       </c>
       <c r="E23" s="7"/>
       <c r="F23" s="7" t="s">
-        <v>943</v>
+        <v>939</v>
       </c>
       <c r="G23" s="7"/>
       <c r="H23" s="7"/>
       <c r="I23" s="7" t="s">
-        <v>944</v>
+        <v>940</v>
       </c>
       <c r="J23" s="7" t="s">
-        <v>945</v>
+        <v>941</v>
       </c>
     </row>
     <row r="24">
@@ -49085,44 +49020,44 @@
       </c>
       <c r="E24" s="7"/>
       <c r="F24" s="7" t="s">
-        <v>946</v>
+        <v>942</v>
       </c>
       <c r="G24" s="7"/>
       <c r="H24" s="7"/>
       <c r="I24" s="7" t="s">
-        <v>947</v>
+        <v>943</v>
       </c>
       <c r="J24" s="6" t="s">
-        <v>948</v>
+        <v>944</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="s">
-        <v>759</v>
+        <v>754</v>
       </c>
       <c r="B25" s="6"/>
       <c r="C25" s="6" t="s">
         <v>116</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>949</v>
+        <v>945</v>
       </c>
       <c r="E25" s="7"/>
       <c r="F25" s="7" t="s">
-        <v>950</v>
+        <v>946</v>
       </c>
       <c r="G25" s="7"/>
       <c r="H25" s="7"/>
       <c r="I25" s="7" t="s">
-        <v>951</v>
+        <v>947</v>
       </c>
       <c r="J25" s="7" t="s">
-        <v>908</v>
+        <v>903</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="s">
-        <v>759</v>
+        <v>754</v>
       </c>
       <c r="B26" s="6"/>
       <c r="C26" s="6" t="s">
@@ -49133,20 +49068,20 @@
       </c>
       <c r="E26" s="7"/>
       <c r="F26" s="7" t="s">
-        <v>952</v>
+        <v>948</v>
       </c>
       <c r="G26" s="7"/>
       <c r="H26" s="7"/>
       <c r="I26" s="7" t="s">
-        <v>953</v>
+        <v>949</v>
       </c>
       <c r="J26" s="7" t="s">
-        <v>954</v>
+        <v>950</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="s">
-        <v>759</v>
+        <v>754</v>
       </c>
       <c r="B27" s="6"/>
       <c r="C27" s="6" t="s">
@@ -49157,20 +49092,20 @@
       </c>
       <c r="E27" s="7"/>
       <c r="F27" s="7" t="s">
-        <v>955</v>
+        <v>951</v>
       </c>
       <c r="G27" s="7"/>
       <c r="H27" s="7"/>
       <c r="I27" s="7" t="s">
-        <v>956</v>
+        <v>952</v>
       </c>
       <c r="J27" s="7" t="s">
-        <v>957</v>
+        <v>953</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="s">
-        <v>759</v>
+        <v>754</v>
       </c>
       <c r="B28" s="6"/>
       <c r="C28" s="6" t="s">
@@ -49181,15 +49116,15 @@
       </c>
       <c r="E28" s="7"/>
       <c r="F28" s="7" t="s">
-        <v>958</v>
+        <v>954</v>
       </c>
       <c r="G28" s="7"/>
       <c r="H28" s="7"/>
       <c r="I28" s="7" t="s">
-        <v>959</v>
+        <v>955</v>
       </c>
       <c r="J28" s="7" t="s">
-        <v>960</v>
+        <v>956</v>
       </c>
     </row>
     <row r="29">
@@ -49205,15 +49140,15 @@
       </c>
       <c r="E29" s="7"/>
       <c r="F29" s="7" t="s">
-        <v>961</v>
+        <v>957</v>
       </c>
       <c r="G29" s="7"/>
       <c r="H29" s="7"/>
       <c r="I29" s="7" t="s">
-        <v>962</v>
+        <v>958</v>
       </c>
       <c r="J29" s="7" t="s">
-        <v>963</v>
+        <v>959</v>
       </c>
     </row>
     <row r="30">
@@ -49229,15 +49164,15 @@
       </c>
       <c r="E30" s="7"/>
       <c r="F30" s="7" t="s">
-        <v>964</v>
+        <v>960</v>
       </c>
       <c r="G30" s="7"/>
       <c r="H30" s="7"/>
       <c r="I30" s="7" t="s">
-        <v>965</v>
+        <v>961</v>
       </c>
       <c r="J30" s="7" t="s">
-        <v>966</v>
+        <v>962</v>
       </c>
     </row>
     <row r="31">
@@ -49253,15 +49188,15 @@
       </c>
       <c r="E31" s="7"/>
       <c r="F31" s="7" t="s">
-        <v>967</v>
+        <v>963</v>
       </c>
       <c r="G31" s="7"/>
       <c r="H31" s="7"/>
       <c r="I31" s="7" t="s">
-        <v>968</v>
+        <v>964</v>
       </c>
       <c r="J31" s="7" t="s">
-        <v>969</v>
+        <v>965</v>
       </c>
     </row>
     <row r="32">
@@ -49277,15 +49212,15 @@
       </c>
       <c r="E32" s="7"/>
       <c r="F32" s="7" t="s">
-        <v>970</v>
+        <v>966</v>
       </c>
       <c r="G32" s="7"/>
       <c r="H32" s="7"/>
       <c r="I32" s="7" t="s">
-        <v>971</v>
+        <v>967</v>
       </c>
       <c r="J32" s="7" t="s">
-        <v>908</v>
+        <v>903</v>
       </c>
     </row>
   </sheetData>

</xml_diff>